<commit_message>
feat: complete fully autonomous weekly PDCA pipeline (insights analysis + idea replenishment + Obsidian sync)
</commit_message>
<xml_diff>
--- a/02_planning/content_ideas_sheet.xlsx
+++ b/02_planning/content_ideas_sheet.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +71,20 @@
       <name val="Helvetica Neue"/>
       <b val="1"/>
       <color rgb="0015803D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Helvetica Neue"/>
+      <color rgb="009CA3AF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Helvetica Neue"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Helvetica Neue"/>
+      <color rgb="004B5563"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -150,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -200,6 +214,14 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -565,8 +587,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -775,6 +797,31 @@
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>〜ておく vs 〜てある (準備と結果の状態)</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>ておく＝事前の準備、てある＝準備された状態が残っている</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -793,8 +840,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -1003,6 +1050,31 @@
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>「とりあえず」のリアルな日常会話の使い方</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>居酒屋での注文、保留、一旦の決定</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -1021,8 +1093,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -1234,6 +1306,31 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>日本到着後の市役所・住民票・国民健康保険手続きガイド</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>スペイン人が最初に行う14日以内の行政手続き</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>